<commit_message>
Batch B: all nine tools, no-AI rules engine, optional AI for Gemini, ChatGPT and Claude
</commit_message>
<xml_diff>
--- a/app/public/sample-data/mousy_batch_20.xlsx
+++ b/app/public/sample-data/mousy_batch_20.xlsx
@@ -572,7 +572,7 @@
 [00:00:41] Customer: no, CANCEL. not a refund
 [00:00:42] Mousy Assist: Sorry, I didn't get that. Could you say it another way?
 [00:00:57] Customer: Hi, I want to cancel my order
-[00:01:00] Mousy Assist: Sure. What's your order number? It looks like MO-1234.
+[00:01:00] Mousy Assist: Sure. What's your order number? It starts with MO.
 [00:01:20] Customer: it's MO-1465
 [00:01:21] Mousy Assist: Thanks. Looking up order MO-1465 now.
 [00:01:23] Mousy Assist: Order MO-1465 has the desk lamp and hasn't shipped yet. Do you want to cancel the whole order?
@@ -1018,7 +1018,7 @@
         <is>
           <t>[00:00:00] Mousy Assist: Hi, I'm Mousy Assist. How can I help with your order today?
 [00:00:15] Customer: the box was crushed and the item is broken
-[00:00:17] Mousy Assist: Sure. What's your order number? It looks like MO-1234.
+[00:00:17] Mousy Assist: Sure. What's your order number? It starts with MO.
 [00:00:30] Customer: MO-4615
 [00:00:31] Mousy Assist: Thanks. Looking up order MO-4615 now.
 [00:00:33] Mousy Assist: I'm sorry it arrived damaged. Order MO-4615 has the desk lamp and the egg timer. Which one is damaged?
@@ -1763,7 +1763,7 @@
         <is>
           <t>[00:00:00] Mousy Assist: Hi, I'm Mousy Assist. How can I help with your order today?
 [00:00:20] Customer: my order still hasn't arrived
-[00:00:22] Mousy Assist: Sure. What's your order number? It looks like MO-1234.
+[00:00:22] Mousy Assist: Sure. What's your order number? It starts with MO.
 [00:00:42] Customer: MO-1021
 [00:00:44] Mousy Assist: Thanks. Looking up order MO-1012 now.
 [00:00:46] Mousy Assist: Order MO-1012 shipped on February 28 with Pawcel Post. It's in Crumbridge and should arrive on Tuesday by 6 pm.

</xml_diff>